<commit_message>
Sync Fair Forward entries with current catalogue
Add 2 datasets newly published in the Fair Forward catalogue since this PR
was opened:
- Our language, our data (DhoNam Dholuo Speech) — Kenya, NLP
- FarmerChat — Kenya; Nigeria; Ethiopia, Agriculture

Reflect upstream name changes by updating titles for entries that were
renamed: Rwanda Media Voice Bridge, the Ltome-Katip biodiversity dataset
(now "Indigenous Knowledge Meets AI..."), and the Kiswahili machine-
translation dataset ("Kenyan" -> "East African" languages). Add East/West
Africa region tags to four existing rows (BenMangroves, the Kiswahili MT
dataset, LivHealth, and the Mozilla Common Voice 3-languages dataset).

Regenerate the Excel mirror so it matches the CSV (296 datasets).
</commit_message>
<xml_diff>
--- a/datasets/Open Datasets and Use Cases Africa.xlsx
+++ b/datasets/Open Datasets and Use Cases Africa.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,68 +413,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J295"/>
+  <dimension ref="A1:J297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="51" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Dataset Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>License</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Use Cases</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Challenges/Notes</t>
         </is>
@@ -13007,7 +12991,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Benin</t>
+          <t>Benin; West Africa</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
@@ -13141,7 +13125,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Ltome-Katip: Pioneering Indigenous-Led Biodiversity Datasets for Ethical AI in Kenya and the Ecuadorian Amazon</t>
+          <t>Indigenous Knowledge Meets AI: Ethical monitoring of climate stress and biodiversity: sounds of elephants and Katip (Ltome-Katip) in Kenya and the Ecuadorian Amazon</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -13707,7 +13691,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Enabling machine translation from Kiswahili into the indigenous Kenyan languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
+          <t>Enabling machine translation from Kiswahili into the indigenous East African languages Kidaw'ida, Kalenjin, and Dholuo, preserving these languages &amp; supporting crowd-sourced voice recognition via Mozilla Common Voice for these languages</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -13724,7 +13708,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya; East Africa</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -13886,7 +13870,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kenya; East Africa</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -14130,7 +14114,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Kenya; Rwanda; Uganda</t>
+          <t>Kenya; Rwanda; Uganda; East Africa</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -15804,7 +15788,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Rwanda Media Voice Bridge</t>
+          <t>Rwanda Media Voice Bridge -  AI-powered voice transcription and translation solution for Rwanda's film and media industry</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -15846,6 +15830,114 @@
       <c r="J295" t="inlineStr">
         <is>
           <t>Fair Forward portfolio. Early stage, functional demo available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Our language, our data: Co-creating equitable governance models with African language communities - language dataset created: Dholuo Speech</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Maseno University (Maseno Centre for Applied Artificial Intelligence), Members from the Dholuo language community 
+Catalyzed by: Mozilla Foundation, FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/)</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Nwulite Obodo Open Data Licence 1.0 (NOODL-1.0)</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://datacollective.mozillafoundation.org/datasets/cmjepxo6t08nmmk07iauvua6v</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>The “DhoNam: Dholuo Speech dataset” is a speech corpus designed to supercharge Automatic Speech Recognition (ASR) and other speech technologies for Dholuo, one of Kenya’s major indigenous languages. This dataset contains native-speaker audio recordings collected through a plat…</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>Fair Forward portfolio. Dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>FarmerChat: Delivering Personalized Farm Advice to 1.6 Million Farmers Across Five Countries</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Powered by / Provided by: Digital Green
+Catalyzed by: FAIR Forward - AI for All (https://www.bmz-digital.global/en/overview-of-initiatives/fair-forward/), GIZ 
+Financed by: BMZ (https://www.bmz-digital.global/en/digital-transformation-and-development-cooperation/) and  Sequoia Climate Fund, CISCO Foundation</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Kenya; Nigeria; Ethiopia</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>CC-BY 4.0</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://github.com/digitalgreenorg/DG_Open</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>FarmerChat is an AI assistant built to help smallholder farmers make better field-level decisions by delivering timely, localized advice to help them grow more, earn more, and adapt to changing weather. It is designed for low-connectivity areas and available in over 15 languag…</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>Fair Forward portfolio. Dataset  &gt; Model &gt; Pilot &gt; Use-Case &gt;  Use-Case with Business Model</t>
         </is>
       </c>
     </row>

</xml_diff>